<commit_message>
feat(content): sync arena content and add video platform support
- Update arena overview content (industrial chain graph, contract legal review)

- Add video play overlay component and platform integration

- Update FAQ, framework, privacy, terms pages with new content

- Enhance xlsx_to_json.py with improved export logic

- Fix .gitignore to include lib directory

- Update translations (en/zh) for new content
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="108">
   <si>
     <t>擂台编号</t>
   </si>
@@ -65,7 +65,16 @@
     <t>攻擂中</t>
   </si>
   <si>
-    <t>视频链接</t>
+    <t>国内视频链接</t>
+  </si>
+  <si>
+    <t>国际视频链接</t>
+  </si>
+  <si>
+    <t>视频封面图片链接</t>
+  </si>
+  <si>
+    <t>首页展示顺序</t>
   </si>
   <si>
     <t>1</t>
@@ -101,7 +110,10 @@
     <t>私部署版：Claude Code +Kimi K2.5/Minimax M2.5/Qwen 3.5 + Metaso</t>
   </si>
   <si>
-    <t>https://rwai-dev.oss-cn-shanghai.aliyuncs.com/1.mov</t>
+    <t>https://www.bilibili.com/video/BV1FxFYzyEk8</t>
+  </si>
+  <si>
+    <t>https://rwai-dev.oss-cn-shanghai.aliyuncs.com/1.JPG</t>
   </si>
   <si>
     <t>2</t>
@@ -135,6 +147,9 @@
   </si>
   <si>
     <t>https://rwai-dev.oss-cn-shanghai.aliyuncs.com/2.mp4</t>
+  </si>
+  <si>
+    <t>https://rwai-dev.oss-cn-shanghai.aliyuncs.com/2.JPG</t>
   </si>
   <si>
     <t>3</t>
@@ -361,13 +376,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -381,6 +389,13 @@
       <color rgb="FF800080"/>
       <name val="等线"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -815,28 +830,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -960,11 +975,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1284,13 +1301,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:P14"/>
   <sheetFormatPr defaultColWidth="9.64285714285714" defaultRowHeight="16.8"/>
   <cols>
-    <col min="1" max="13" width="19" customWidth="1"/>
+    <col min="1" max="11" width="19" customWidth="1"/>
+    <col min="12" max="12" width="94.7857142857143" customWidth="1"/>
+    <col min="13" max="16" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13" customHeight="1" spans="1:13">
+    <row r="1" ht="13" customHeight="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1330,505 +1349,536 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" ht="25.5" customHeight="1" spans="1:13">
+    <row r="2" ht="25.5" customHeight="1" spans="1:16">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" t="s">
+        <v>28</v>
+      </c>
+      <c r="P2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" t="s">
+        <v>35</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+      <c r="J3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" t="s">
+        <v>25</v>
+      </c>
+      <c r="L3" t="s">
+        <v>38</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="O3" t="s">
+        <v>40</v>
+      </c>
+      <c r="P3" t="s">
         <v>16</v>
       </c>
-      <c r="E2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
+    </row>
+    <row r="4" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" t="s">
         <v>19</v>
       </c>
-      <c r="H2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" t="s">
+        <v>47</v>
+      </c>
+      <c r="N4" s="3"/>
+      <c r="P4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F5" t="s">
         <v>21</v>
       </c>
-      <c r="J2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="G5" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" t="s">
+        <v>53</v>
+      </c>
+      <c r="J5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" t="s">
+        <v>53</v>
+      </c>
+      <c r="J6" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F7" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7" t="s">
+        <v>67</v>
+      </c>
+      <c r="H7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" t="s">
+        <v>53</v>
+      </c>
+      <c r="J7" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" t="s">
         <v>22</v>
       </c>
-      <c r="L2" t="s">
+      <c r="H8" t="s">
         <v>23</v>
       </c>
-      <c r="M2" t="s">
+      <c r="I8" t="s">
+        <v>53</v>
+      </c>
+      <c r="J8" t="s">
         <v>24</v>
       </c>
+      <c r="K8" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" t="s">
+        <v>68</v>
+      </c>
     </row>
-    <row r="3" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A3" t="s">
+    <row r="9" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" t="s">
+        <v>79</v>
+      </c>
+      <c r="H9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I9" t="s">
+        <v>53</v>
+      </c>
+      <c r="J9" t="s">
+        <v>24</v>
+      </c>
+      <c r="K9" t="s">
         <v>25</v>
       </c>
-      <c r="B3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J3" t="s">
-        <v>33</v>
-      </c>
-      <c r="K3" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" t="s">
-        <v>34</v>
-      </c>
-      <c r="M3" t="s">
-        <v>35</v>
+      <c r="L9" t="s">
+        <v>68</v>
       </c>
     </row>
-    <row r="4" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" t="s">
+    <row r="10" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" t="s">
+        <v>76</v>
+      </c>
+      <c r="E10" t="s">
+        <v>83</v>
+      </c>
+      <c r="F10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" t="s">
+        <v>85</v>
+      </c>
+      <c r="H10" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" t="s">
+        <v>53</v>
+      </c>
+      <c r="J10" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" t="s">
+        <v>89</v>
+      </c>
+      <c r="F11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" t="s">
+        <v>60</v>
+      </c>
+      <c r="H11" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" t="s">
+        <v>24</v>
+      </c>
+      <c r="J11" t="s">
+        <v>24</v>
+      </c>
+      <c r="K11" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" t="s">
+        <v>94</v>
+      </c>
+      <c r="D12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" t="s">
+        <v>95</v>
+      </c>
+      <c r="F12" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" t="s">
+        <v>97</v>
+      </c>
+      <c r="H12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" t="s">
         <v>37</v>
       </c>
-      <c r="C4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>39</v>
-      </c>
-      <c r="F4" t="s">
-        <v>40</v>
-      </c>
-      <c r="G4" t="s">
-        <v>41</v>
-      </c>
-      <c r="H4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" t="s">
-        <v>21</v>
-      </c>
-      <c r="K4" t="s">
-        <v>22</v>
-      </c>
-      <c r="L4" t="s">
-        <v>42</v>
+      <c r="J12" t="s">
+        <v>24</v>
+      </c>
+      <c r="K12" t="s">
+        <v>25</v>
+      </c>
+      <c r="L12" t="s">
+        <v>98</v>
       </c>
     </row>
-    <row r="5" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C5" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" t="s">
+    <row r="13" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A13" t="s">
+        <v>99</v>
+      </c>
+      <c r="B13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" t="s">
+        <v>101</v>
+      </c>
+      <c r="D13" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" t="s">
+        <v>102</v>
+      </c>
+      <c r="F13" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" t="s">
+        <v>97</v>
+      </c>
+      <c r="H13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" t="s">
+        <v>53</v>
+      </c>
+      <c r="J13" t="s">
+        <v>24</v>
+      </c>
+      <c r="K13" t="s">
+        <v>25</v>
+      </c>
+      <c r="L13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" ht="25.5" customHeight="1" spans="1:16">
+      <c r="A14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" t="s">
+        <v>105</v>
+      </c>
+      <c r="C14" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" t="s">
+        <v>106</v>
+      </c>
+      <c r="F14" t="s">
+        <v>107</v>
+      </c>
+      <c r="G14" t="s">
+        <v>97</v>
+      </c>
+      <c r="H14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" t="s">
+        <v>53</v>
+      </c>
+      <c r="J14" t="s">
+        <v>24</v>
+      </c>
+      <c r="K14" t="s">
+        <v>25</v>
+      </c>
+      <c r="L14" t="s">
         <v>47</v>
-      </c>
-      <c r="H5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I5" t="s">
-        <v>48</v>
-      </c>
-      <c r="J5" t="s">
-        <v>21</v>
-      </c>
-      <c r="K5" t="s">
-        <v>22</v>
-      </c>
-      <c r="L5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" t="s">
-        <v>54</v>
-      </c>
-      <c r="G6" t="s">
-        <v>55</v>
-      </c>
-      <c r="H6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" t="s">
-        <v>48</v>
-      </c>
-      <c r="J6" t="s">
-        <v>21</v>
-      </c>
-      <c r="K6" t="s">
-        <v>22</v>
-      </c>
-      <c r="L6" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B7" t="s">
-        <v>58</v>
-      </c>
-      <c r="C7" t="s">
-        <v>59</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7" t="s">
-        <v>61</v>
-      </c>
-      <c r="G7" t="s">
-        <v>62</v>
-      </c>
-      <c r="H7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" t="s">
-        <v>48</v>
-      </c>
-      <c r="J7" t="s">
-        <v>21</v>
-      </c>
-      <c r="K7" t="s">
-        <v>22</v>
-      </c>
-      <c r="L7" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A8" t="s">
-        <v>64</v>
-      </c>
-      <c r="B8" t="s">
-        <v>65</v>
-      </c>
-      <c r="C8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" t="s">
-        <v>67</v>
-      </c>
-      <c r="F8" t="s">
-        <v>29</v>
-      </c>
-      <c r="G8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" t="s">
-        <v>48</v>
-      </c>
-      <c r="J8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="9" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" t="s">
-        <v>72</v>
-      </c>
-      <c r="F9" t="s">
-        <v>73</v>
-      </c>
-      <c r="G9" t="s">
-        <v>74</v>
-      </c>
-      <c r="H9" t="s">
-        <v>31</v>
-      </c>
-      <c r="I9" t="s">
-        <v>48</v>
-      </c>
-      <c r="J9" t="s">
-        <v>21</v>
-      </c>
-      <c r="K9" t="s">
-        <v>22</v>
-      </c>
-      <c r="L9" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="10" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A10" t="s">
-        <v>75</v>
-      </c>
-      <c r="B10" t="s">
-        <v>76</v>
-      </c>
-      <c r="C10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" t="s">
-        <v>71</v>
-      </c>
-      <c r="E10" t="s">
-        <v>78</v>
-      </c>
-      <c r="F10" t="s">
-        <v>79</v>
-      </c>
-      <c r="G10" t="s">
-        <v>80</v>
-      </c>
-      <c r="H10" t="s">
-        <v>20</v>
-      </c>
-      <c r="I10" t="s">
-        <v>48</v>
-      </c>
-      <c r="J10" t="s">
-        <v>21</v>
-      </c>
-      <c r="K10" t="s">
-        <v>22</v>
-      </c>
-      <c r="L10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="11" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A11" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" t="s">
-        <v>82</v>
-      </c>
-      <c r="C11" t="s">
-        <v>83</v>
-      </c>
-      <c r="D11" t="s">
-        <v>71</v>
-      </c>
-      <c r="E11" t="s">
-        <v>84</v>
-      </c>
-      <c r="F11" t="s">
-        <v>85</v>
-      </c>
-      <c r="G11" t="s">
-        <v>55</v>
-      </c>
-      <c r="H11" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" t="s">
-        <v>21</v>
-      </c>
-      <c r="J11" t="s">
-        <v>21</v>
-      </c>
-      <c r="K11" t="s">
-        <v>48</v>
-      </c>
-      <c r="L11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A12" t="s">
-        <v>87</v>
-      </c>
-      <c r="B12" t="s">
-        <v>88</v>
-      </c>
-      <c r="C12" t="s">
-        <v>89</v>
-      </c>
-      <c r="D12" t="s">
-        <v>71</v>
-      </c>
-      <c r="E12" t="s">
-        <v>90</v>
-      </c>
-      <c r="F12" t="s">
-        <v>91</v>
-      </c>
-      <c r="G12" t="s">
-        <v>92</v>
-      </c>
-      <c r="H12" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" t="s">
-        <v>33</v>
-      </c>
-      <c r="J12" t="s">
-        <v>21</v>
-      </c>
-      <c r="K12" t="s">
-        <v>22</v>
-      </c>
-      <c r="L12" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="13" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A13" t="s">
-        <v>94</v>
-      </c>
-      <c r="B13" t="s">
-        <v>95</v>
-      </c>
-      <c r="C13" t="s">
-        <v>96</v>
-      </c>
-      <c r="D13" t="s">
-        <v>71</v>
-      </c>
-      <c r="E13" t="s">
-        <v>97</v>
-      </c>
-      <c r="F13" t="s">
-        <v>73</v>
-      </c>
-      <c r="G13" t="s">
-        <v>92</v>
-      </c>
-      <c r="H13" t="s">
-        <v>20</v>
-      </c>
-      <c r="I13" t="s">
-        <v>48</v>
-      </c>
-      <c r="J13" t="s">
-        <v>21</v>
-      </c>
-      <c r="K13" t="s">
-        <v>22</v>
-      </c>
-      <c r="L13" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="14" ht="25.5" customHeight="1" spans="1:13">
-      <c r="A14" t="s">
-        <v>99</v>
-      </c>
-      <c r="B14" t="s">
-        <v>100</v>
-      </c>
-      <c r="C14" t="s">
-        <v>96</v>
-      </c>
-      <c r="D14" t="s">
-        <v>71</v>
-      </c>
-      <c r="E14" t="s">
-        <v>101</v>
-      </c>
-      <c r="F14" t="s">
-        <v>102</v>
-      </c>
-      <c r="G14" t="s">
-        <v>92</v>
-      </c>
-      <c r="H14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I14" t="s">
-        <v>48</v>
-      </c>
-      <c r="J14" t="s">
-        <v>21</v>
-      </c>
-      <c r="K14" t="s">
-        <v>22</v>
-      </c>
-      <c r="L14" t="s">
-        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -1849,6 +1899,12 @@
       <formula1>"较优,中等"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="M2" r:id="rId1" display="https://www.bilibili.com/video/BV1FxFYzyEk8"/>
+    <hyperlink ref="N2" r:id="rId1" display="https://www.bilibili.com/video/BV1FxFYzyEk8"/>
+    <hyperlink ref="M3" r:id="rId2" display="https://rwai-dev.oss-cn-shanghai.aliyuncs.com/2.mp4"/>
+    <hyperlink ref="N3" r:id="rId2" display="https://rwai-dev.oss-cn-shanghai.aliyuncs.com/2.mp4"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
refactor(arena): move related references to overview and remove video covers
- Remove video cover image URLs for arenas 1 and 2
- Parse related references as clickable links in overview section
- Remove related references phase from implementation section

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -507,11 +507,7 @@
           <t>https://www.bilibili.com/video/BV1FxFYzyEk8</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>https://rwai-dev.oss-cn-shanghai.aliyuncs.com/1.JPG</t>
-        </is>
-      </c>
+      <c r="P2"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>2</t>
@@ -596,11 +592,7 @@
           <t>https://www.bilibili.com/video/BV1qxwXzAEME</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>https://rwai-dev.oss-cn-shanghai.aliyuncs.com/2.JPG</t>
-        </is>
-      </c>
+      <c r="P3"/>
       <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>

</xml_diff>

<commit_message>
feat(content): add BISHENG GitHub reference for arena 8
- Add BISHENG GitHub link to arena 8 related references
- Update CSV, Excel, and JSON data files

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -986,7 +986,11 @@
           <t>私部署版：BISHENG</t>
         </is>
       </c>
-      <c r="D9"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BISHENG GitHub：https://github.com/dataelement/bisheng</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>验证中</t>

</xml_diff>

<commit_message>
chore(content): update arena data for 2026-05-18 and upgrade intelligent-research-system deps
- Update review dates from 2026-05-11 to 2026-05-18 across all arenas
- Remove "最近审阅" field from arena metadata (main.md, overview, raw.json)
- Upgrade intelligent-research-system: Metaso MCP → StepSearch MCP, GLM-5 → DeepSeek V4 Pro
- Update DeepResearch Bench score from 51.86 (rank 2) to 53.54 (rank 3)
- Add StepSearch MCP configuration step to tech-configuration docs

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content/Arena/List of Arenas.xlsx
+++ b/Content/Arena/List of Arenas.xlsx
@@ -442,14 +442,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + GLM 5 + Metaso</t>
+          <t>私部署版：Claude Code + DeepSeek V4 Pro + StepSearch</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Claude Code (by Anthropic) GitHub：https://github.com/anthropics/claude-code
-Metaso MCP (by 秘塔科技) 文档：https://www.modelscope.cn/mcp/servers/metasota/metaso-search
-GLM-5(by 智谱) GitHub：https://github.com/zai-org/GLM-5</t>
+StepSearch MCP (by 阶跃星辰) 文档：https://platform.stepfun.com/docs/zh/step-plan/integrations/search-mcp
+DeepSeek-V4-Pro(by 深度求索) Hugging Face：https://huggingface.co/deepseek-ai/DeepSeek-V4-Pro</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -494,7 +494,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>私部署版：Claude Code + DeepSeek V4 Pro/MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6+ Metaso</t>
+          <t>私部署版：Hermes Agent + MiMo V2.5 Pro/GLM 5.1/Kimi K2.6/Qwen 3.6+ Metaso</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">

</xml_diff>